<commit_message>
Sección equipo y ubicación dinámicas desde Excel, mapa interactivo con Folium
</commit_message>
<xml_diff>
--- a/directorio_casas_juventud.xlsx
+++ b/directorio_casas_juventud.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carol\CH_projects\SDIS\Gestion de conocimiento\gestor-conocimiento-2025\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AE5A21E-42C3-4192-88DC-D8D96C5EE3E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -250,8 +256,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="178" formatCode="0.0000000000000"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -259,16 +268,36 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -276,25 +305,55 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="178" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="178" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -332,7 +391,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -366,6 +425,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -400,9 +460,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -575,408 +636,418 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H20"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="34.86328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.46484375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30.3984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.06640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.73046875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" t="s">
+    <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="E2">
-        <v>4.586325</v>
-      </c>
-      <c r="F2">
-        <v>-74.099996</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" t="s">
+      <c r="E2" s="7">
+        <v>4.5851577074113896</v>
+      </c>
+      <c r="F2" s="7">
+        <v>-74.103246468893303</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="E3">
-        <v>4.663042</v>
-      </c>
-      <c r="F3">
-        <v>-74.064919</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" t="s">
+      <c r="E3" s="7">
+        <v>4.6689440006099003</v>
+      </c>
+      <c r="F3" s="7">
+        <v>-74.077943787523495</v>
+      </c>
+      <c r="H3" s="3"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="E4">
-        <v>4.611104</v>
-      </c>
-      <c r="F4">
-        <v>-74.19358</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
+      <c r="E4" s="7">
+        <v>4.6127386710881702</v>
+      </c>
+      <c r="F4" s="7">
+        <v>-74.193902501018101</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="E5">
-        <v>4.5942</v>
-      </c>
-      <c r="F5">
-        <v>-74.069371</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" t="s">
+      <c r="E5" s="7">
+        <v>4.59287910555281</v>
+      </c>
+      <c r="F5" s="7">
+        <v>-74.069944935161502</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="E6">
-        <v>4.6494</v>
-      </c>
-      <c r="F6">
-        <v>-74.0628</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" t="s">
+      <c r="E6" s="7">
+        <v>4.6466963500016902</v>
+      </c>
+      <c r="F6" s="7">
+        <v>-74.054178481485096</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A7" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="E7">
-        <v>4.5694</v>
-      </c>
-      <c r="F7">
-        <v>-74.1558</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" t="s">
+      <c r="E7" s="7">
+        <v>4.5529030850434697</v>
+      </c>
+      <c r="F7" s="7">
+        <v>-74.139195919818505</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="E8">
-        <v>4.585557</v>
-      </c>
-      <c r="F8">
-        <v>-74.156869</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" t="s">
+      <c r="E8" s="7">
+        <v>4.5513769205001102</v>
+      </c>
+      <c r="F8" s="7">
+        <v>-74.162166277490002</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A9" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="E9">
-        <v>4.693314</v>
-      </c>
-      <c r="F9">
-        <v>-74.110938</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" t="s">
+      <c r="E9" s="7">
+        <v>4.6947199091824299</v>
+      </c>
+      <c r="F9" s="7">
+        <v>-74.109543717967796</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A10" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="E10">
-        <v>4.681777</v>
-      </c>
-      <c r="F10">
-        <v>-74.12152500000001</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" t="s">
+      <c r="E10" s="7">
+        <v>4.6850170786969096</v>
+      </c>
+      <c r="F10" s="7">
+        <v>-74.156304182385796</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A11" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="E11">
-        <v>4.616364</v>
-      </c>
-      <c r="F11">
-        <v>-74.16598</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" t="s">
+      <c r="E11" s="5">
+        <v>4.6236509738103297</v>
+      </c>
+      <c r="F11" s="5">
+        <v>-74.156251390982604</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A12" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="E12">
-        <v>4.615032</v>
-      </c>
-      <c r="F12">
-        <v>-74.083249</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
-      <c r="A13" t="s">
+      <c r="E12" s="5">
+        <v>4.6227331619645602</v>
+      </c>
+      <c r="F12" s="5">
+        <v>-74.081139060296394</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A13" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="E13">
-        <v>4.5615</v>
-      </c>
-      <c r="F13">
-        <v>-74.11450000000001</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" t="s">
+      <c r="E13" s="5">
+        <v>4.5515216705112298</v>
+      </c>
+      <c r="F13" s="5">
+        <v>-74.109366760296595</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A14" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="E14">
-        <v>4.568741</v>
-      </c>
-      <c r="F14">
-        <v>-74.087504</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" t="s">
+      <c r="E14" s="5">
+        <v>4.5762453547997204</v>
+      </c>
+      <c r="F14" s="5">
+        <v>-74.0824997875267</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A15" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="E15">
-        <v>4.741396</v>
-      </c>
-      <c r="F15">
-        <v>-74.112996</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" t="s">
+      <c r="E15" s="5">
+        <v>4.7411755826625503</v>
+      </c>
+      <c r="F15" s="5">
+        <v>-74.108112775639199</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A16" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="E16">
-        <v>4.51737</v>
-      </c>
-      <c r="F16">
-        <v>-74.115571</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6">
-      <c r="A17" t="s">
+      <c r="E16" s="5">
+        <v>4.5124085761856101</v>
+      </c>
+      <c r="F16" s="5">
+        <v>-74.114615635161499</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A17" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="E17">
-        <v>4.601412</v>
-      </c>
-      <c r="F17">
-        <v>-74.10719899999999</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6">
-      <c r="A18" t="s">
+      <c r="E17" s="5">
+        <v>4.6036850029466203</v>
+      </c>
+      <c r="F17" s="5">
+        <v>-74.105577204475395</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A18" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="E18">
-        <v>4.577265</v>
-      </c>
-      <c r="F18">
-        <v>-74.16689700000001</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6">
-      <c r="A19" t="s">
+      <c r="E18" s="5">
+        <v>4.5771220701844699</v>
+      </c>
+      <c r="F18" s="5">
+        <v>-74.166916680596202</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A19" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="E19">
-        <v>4.593173</v>
-      </c>
-      <c r="F19">
-        <v>-74.139385</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="A20" t="s">
+      <c r="E19" s="5">
+        <v>4.5852218744055104</v>
+      </c>
+      <c r="F19" s="5">
+        <v>-74.103284019818503</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A20" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="E20">
-        <v>4.731695</v>
-      </c>
-      <c r="F20">
-        <v>-74.029291</v>
+      <c r="E20" s="5">
+        <v>4.7342311274868196</v>
+      </c>
+      <c r="F20" s="5">
+        <v>-74.025570338939303</v>
       </c>
     </row>
   </sheetData>

</xml_diff>